<commit_message>
fix: align excel tracker column names to prevent duplicate columns during pandas append
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker.xlsx
+++ b/Job_Application_Tracker.xlsx
@@ -19,50 +19,50 @@
     <t>公司 (Company)</t>
   </si>
   <si>
-    <t>岗位名称 (Role)</t>
-  </si>
-  <si>
-    <t>投递状态 (Status)</t>
-  </si>
-  <si>
-    <t>核心关键词 (Keywords)</t>
-  </si>
-  <si>
-    <t>完整JD/链接 (JD Link)</t>
-  </si>
-  <si>
-    <t>使用简历版本 (Resume Used)</t>
-  </si>
-  <si>
-    <t>投递时间 (Date)</t>
+    <t>部门 (Department)</t>
+  </si>
+  <si>
+    <t>岗位 (Role)</t>
+  </si>
+  <si>
+    <t>JD链接/核心要求 (JD Link / Core Reqs)</t>
+  </si>
+  <si>
+    <t>投递时间 (Apply Date)</t>
+  </si>
+  <si>
+    <t>发现及投递渠道 (Channel)</t>
+  </si>
+  <si>
+    <t>使用的简历版本 (Resume Version)</t>
+  </si>
+  <si>
+    <t>当前状态 (Current Status)</t>
+  </si>
+  <si>
+    <t>笔试/测评 (Assessment)</t>
+  </si>
+  <si>
+    <t>一面时间 (1st Interview)</t>
+  </si>
+  <si>
+    <t>二面时间 (2nd Interview)</t>
+  </si>
+  <si>
+    <t>HR面/终面 (Final Interview)</t>
+  </si>
+  <si>
+    <t>复盘与备注 (Notes)</t>
   </si>
   <si>
     <t>示例公司</t>
-  </si>
-  <si>
-    <t>AI产品经理</t>
-  </si>
-  <si>
-    <t>已投递</t>
-  </si>
-  <si>
-    <t>生态构建、数据驱动</t>
-  </si>
-  <si>
-    <t>https://example.com/jd</t>
-  </si>
-  <si>
-    <t>review_draft_示例_AI.md</t>
-  </si>
-  <si>
-    <t>2026-05-17</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -77,13 +77,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -118,22 +111,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -426,10 +413,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -451,34 +438,31 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>